<commit_message>
Backlog e Historias de Usuario
</commit_message>
<xml_diff>
--- a/Proyecto-Eventual/1. Elicitación/1.1 Cronograma/Cronograma_Actividades_v.1.1.xlsx
+++ b/Proyecto-Eventual/1. Elicitación/1.1 Cronograma/Cronograma_Actividades_v.1.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\6to semestre\Analisi y diseño\AlexCuzco_30724_G5_ADSW\Proyecto-Eventual\1. Elicitación\1.1 Cronograma\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39594B8-68F3-48C4-B3AC-6C89E35E73F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E655608-8D17-495F-B208-76A559CA5600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="37">
   <si>
     <t>ID Tarea</t>
   </si>
@@ -138,9 +138,6 @@
   </si>
   <si>
     <t>RF02 - Gestionar Miembros, Diagramas de secuencia</t>
-  </si>
-  <si>
-    <t>Backlog Version 1, Historias de usuario</t>
   </si>
   <si>
     <t>RF03 - Consultar calendario de eventos, Diagrama de secuancias, Matriz IREB 3 Requisitos</t>
@@ -772,7 +769,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>27</v>
@@ -856,7 +853,7 @@
         <v>11</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>26</v>
@@ -880,24 +877,24 @@
       <c r="O8" s="11"/>
     </row>
     <row r="9" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B9" s="2"/>
+      <c r="B9" s="22" t="s">
+        <v>12</v>
+      </c>
       <c r="C9" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>6</v>
+        <v>18</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="21" t="s">
+        <v>30</v>
       </c>
       <c r="F9" s="5">
-        <v>46151</v>
+        <v>46156</v>
       </c>
       <c r="G9" s="17">
-        <v>46155</v>
+        <v>46164</v>
       </c>
       <c r="H9" s="19"/>
-      <c r="I9" s="25"/>
+      <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
       <c r="L9" s="11"/>
@@ -907,10 +904,10 @@
     </row>
     <row r="10" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="B10" s="22" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="21" t="s">
@@ -933,10 +930,10 @@
     </row>
     <row r="11" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="B11" s="22" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D11" s="3"/>
       <c r="E11" s="21" t="s">
@@ -959,10 +956,10 @@
     </row>
     <row r="12" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="B12" s="22" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="21" t="s">
@@ -985,20 +982,20 @@
     </row>
     <row r="13" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="B13" s="22" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D13" s="3"/>
       <c r="E13" s="21" t="s">
         <v>30</v>
       </c>
       <c r="F13" s="5">
-        <v>46156</v>
+        <v>46165</v>
       </c>
       <c r="G13" s="17">
-        <v>46164</v>
+        <v>46173</v>
       </c>
       <c r="H13" s="19"/>
       <c r="I13" s="19"/>
@@ -1011,10 +1008,10 @@
     </row>
     <row r="14" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
       <c r="B14" s="22" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" s="3"/>
       <c r="E14" s="21" t="s">
@@ -1036,13 +1033,13 @@
       <c r="O14" s="11"/>
     </row>
     <row r="15" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B15" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D15" s="3"/>
+      <c r="B15" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="6"/>
       <c r="E15" s="21" t="s">
         <v>30</v>
       </c>
@@ -1052,23 +1049,23 @@
       <c r="G15" s="17">
         <v>46173</v>
       </c>
-      <c r="H15" s="19"/>
-      <c r="I15" s="19"/>
-      <c r="J15" s="19"/>
-      <c r="K15" s="19"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
       <c r="L15" s="11"/>
       <c r="M15" s="11"/>
       <c r="N15" s="11"/>
       <c r="O15" s="11"/>
     </row>
     <row r="16" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B16" s="23" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="D16" s="6"/>
+      <c r="B16" s="24" t="s">
+        <v>31</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="12"/>
       <c r="E16" s="21" t="s">
         <v>30</v>
       </c>
@@ -1078,36 +1075,26 @@
       <c r="G16" s="17">
         <v>46173</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="19"/>
+      <c r="J16" s="19"/>
+      <c r="K16" s="19"/>
       <c r="L16" s="11"/>
       <c r="M16" s="11"/>
       <c r="N16" s="11"/>
       <c r="O16" s="11"/>
     </row>
     <row r="17" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B17" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="D17" s="12"/>
-      <c r="E17" s="21" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17" s="5">
-        <v>46165</v>
-      </c>
-      <c r="G17" s="17">
-        <v>46173</v>
-      </c>
-      <c r="H17" s="19"/>
-      <c r="I17" s="19"/>
-      <c r="J17" s="19"/>
-      <c r="K17" s="19"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
       <c r="L17" s="11"/>
       <c r="M17" s="11"/>
       <c r="N17" s="11"/>
@@ -1337,17 +1324,7 @@
       <c r="N31" s="11"/>
       <c r="O31" s="11"/>
     </row>
-    <row r="32" spans="2:15" ht="16.5" x14ac:dyDescent="0.45">
-      <c r="B32" s="7"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="9"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="11"/>
-      <c r="I32" s="11"/>
-      <c r="J32" s="11"/>
-      <c r="K32" s="11"/>
+    <row r="32" spans="2:15" x14ac:dyDescent="0.35">
       <c r="L32" s="11"/>
       <c r="M32" s="11"/>
       <c r="N32" s="11"/>

</xml_diff>